<commit_message>
Update architecture image assets
</commit_message>
<xml_diff>
--- a/images_generator/graphic_image/data.xlsx
+++ b/images_generator/graphic_image/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chpsv\Documents\MPEngEletrica\Master Project\LiteML\trainings\image\imagens_graficas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chpsv\Documents\MPEngEletrica\Master Project\LiteML\utils\image_generator\graphic_image\x\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4803BC7-4FA4-4B4F-BF9C-E8B2669B38B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34A470F-B02F-4253-ADC8-6ADDC88A7162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DAD1E0F3-1F5C-4F05-B6BF-774D712084D6}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>H_p</t>
   </si>
   <si>
-    <t>Predictions_rolling24_MLP_Python</t>
-  </si>
-  <si>
     <t>window_start</t>
   </si>
   <si>
@@ -95,9 +92,6 @@
     <t>R2_H</t>
   </si>
   <si>
-    <t>Metrics_rolling24_MLP_Python</t>
-  </si>
-  <si>
     <t>Tin</t>
   </si>
   <si>
@@ -107,13 +101,19 @@
     <t>Hp</t>
   </si>
   <si>
-    <t>Predictions_rolling24_MLP_Firmware_Replay</t>
-  </si>
-  <si>
-    <t>Metrics_rolling24_MLP_Firmware_Replay</t>
-  </si>
-  <si>
     <t>2019-01-05 05:00:00</t>
+  </si>
+  <si>
+    <t>Metrics_rolling24_Conv1D_Tiny_Python</t>
+  </si>
+  <si>
+    <t>Predictions_rolling24_Conv1D_Tiny_Python</t>
+  </si>
+  <si>
+    <t>Predictions_rolling24_Conv1D_Tiny_Firmware_Replay</t>
+  </si>
+  <si>
+    <t>Metrics_rolling24_Conv1D_Tiny_Firmware_Replay</t>
   </si>
 </sst>
 </file>
@@ -594,20 +594,20 @@
   <cols>
     <col min="1" max="1" width="12.26953125" customWidth="1"/>
     <col min="2" max="3" width="9.6328125" customWidth="1"/>
-    <col min="4" max="4" width="10.90625" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" customWidth="1"/>
     <col min="7" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="17.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
       <c r="D1" s="8"/>
       <c r="G1" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
@@ -636,43 +636,43 @@
         <v>3</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
@@ -695,7 +695,7 @@
         <v>1981</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J3" s="4">
         <v>24</v>
@@ -1052,13 +1052,13 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="G28" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
@@ -1075,55 +1075,55 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G29" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H29" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="I29" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I29" s="3" t="s">
+      <c r="J29" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J29" s="3" t="s">
+      <c r="K29" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="L29" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L29" s="3" t="s">
+      <c r="M29" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M29" s="3" t="s">
+      <c r="N29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N29" s="3" t="s">
+      <c r="O29" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O29" s="3" t="s">
+      <c r="P29" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P29" s="3" t="s">
+      <c r="Q29" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q29" s="3" t="s">
+      <c r="R29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R29" s="3" t="s">
+      <c r="S29" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="S29" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.35">
@@ -1146,7 +1146,7 @@
         <v>1981</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J30" s="4">
         <v>24</v>

</xml_diff>